<commit_message>
audit(2026-06-18): update PRs sheet with PR #215 link
</commit_message>
<xml_diff>
--- a/audits/daily_usability_audit_2026-06-18.xlsx
+++ b/audits/daily_usability_audit_2026-06-18.xlsx
@@ -58,7 +58,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +89,12 @@
         <bgColor rgb="00E5E7EB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -116,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +146,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12012,34 +12021,34 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>funder-finder / fundermatch.org</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>No usability fixes required today (full pass)</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>FM-*, FM-LM-*, FM-IC-* all pass</t>
-        </is>
-      </c>
-      <c r="F4" s="10" t="inlineStr">
-        <is>
-          <t>skip</t>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>audit/2026-06-18-usability</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>#215</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>audit(2026-06-18): daily usability audit report — committed to funder-finder</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="inlineStr">
+        <is>
+          <t>Audit deliverable (no usability fixes required)</t>
+        </is>
+      </c>
+      <c r="F4" s="11" t="inlineStr">
+        <is>
+          <t>open</t>
         </is>
       </c>
     </row>

</xml_diff>